<commit_message>
update meta data and remove maxfill
</commit_message>
<xml_diff>
--- a/automation/badi_aktuell_crowdmonitor/meta_ssd_badi_aktuell.xlsx
+++ b/automation/badi_aktuell_crowdmonitor/meta_ssd_badi_aktuell.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\OGD_Dropzone\INT_DWH\ssd_spo_badi_aktuell\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sszgua\git\opendatazurich.github.io\automation\badi_aktuell_crowdmonitor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771CB04B-1A2A-4D06-A0DA-8345A028B45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A83FE9DE-CE89-4870-8B1E-49DDE2BF2352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="5700" windowWidth="19785" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="14" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="190">
   <si>
     <t>Tagname</t>
   </si>
@@ -978,12 +978,6 @@
     <t>ID des Standorts</t>
   </si>
   <si>
-    <t>Eindeute ID des Standorts</t>
-  </si>
-  <si>
-    <t>Sprechender Name des Standorts</t>
-  </si>
-  <si>
     <t>Anzahl Gäste</t>
   </si>
   <si>
@@ -1020,14 +1014,23 @@
     <t>Detaillierte Informationen finden Sie auf der Webseite [Badi aktuell](https://www.stadt-zuerich.ch/badi-aktuell).</t>
   </si>
   <si>
-    <t>Enthalten sind jene Hallen- und Sommerbäder, die vom Sportamt betrieben werden. Einige Fremdbetriebene Bäder (Dolder, Schanzengraben), Gratisbäder und Bäder im Umbau werden nicht aufgeführt.</t>
-  </si>
-  <si>
     <t>Datenerhebung:</t>
   </si>
   <si>
-    <t>Die dargestellten Zahlen stammen direkt von den Sensoren, die in der Nähe der Kassen aufgestellt sind. Die Sensordaten entsprechen nicht genau den bezahlten Eintritten. Erfahrungsgemäss sind die Sensordaten etwa 20 % höher als die bezahlten Eintritte. Das liegt daran, dass die Sensoren auch weiterzählen, wenn z. B. Kinder im Kassenbereich hin und her laufen.
+    <t>Die dargestellten Zahlen stammen direkt von den Sensoren, die in der Nähe der Kassen aufgestellt sind. Die Sensordaten entsprechen nicht genau den Eintritten. Erfahrungsgemäss sind die Sensordaten etwa 20 % höher als die Eintritte. Das liegt daran, dass die Sensoren mehrfach zählen, wenn Personen das Bad verlassen und wieder betreten oder wenn z. B. Kinder im Kassenbereich hin und herlaufen.
 Die Sensoren bleiben im Winterbetrieb aktiv.</t>
+  </si>
+  <si>
+    <t>Enthalten sind jene Hallen- und Freibäder, die vom Sportamt betrieben werden. In einigen fremdbetriebene Bädern (Dolder, Schanzengraben), Gratisbäder und Bäder im Umbau werden keine Daten erfasst und sie sind darum nicht aufgeführt.</t>
+  </si>
+  <si>
+    <t>occupancy_icons</t>
+  </si>
+  <si>
+    <t>Auslastung</t>
+  </si>
+  <si>
+    <t>Schematische Darstellung der Auslastung mit Icons (entspricht der Auslastungsanzeige auf https://www.stadt-zuerich.ch/badi-aktuell)</t>
   </si>
 </sst>
 </file>
@@ -1795,7 +1798,7 @@
         <v>9</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="7" t="s">
@@ -1813,7 +1816,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="33" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="8" t="s">
@@ -2120,7 +2123,7 @@
         <v>162</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="7"/>
@@ -2133,10 +2136,10 @@
         <v>62</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="7"/>
@@ -2146,10 +2149,10 @@
         <v>62</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="7"/>
@@ -2204,10 +2207,10 @@
         <v>170</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="4" t="s">
@@ -2222,10 +2225,10 @@
         <v>167</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="4" t="s">
@@ -2240,25 +2243,23 @@
         <v>169</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="11" t="s">
-        <v>72</v>
-      </c>
+      <c r="A31" s="11"/>
       <c r="B31" s="20" t="s">
         <v>168</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E31" s="7"/>
     </row>
@@ -2273,15 +2274,23 @@
         <v>171</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E32" s="7"/>
     </row>
-    <row r="33" spans="1:5" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="7"/>
+    <row r="33" spans="1:5" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A33" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>189</v>
+      </c>
       <c r="E33" s="7"/>
     </row>
     <row r="34" spans="1:5" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -2874,26 +2883,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="637d3f4c-beee-42dd-a17b-93f7589025e5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="31d8624d-d3e1-4449-addd-518bfa42d279">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010036EB69643BC4D84A90CF31D6917ED8B0" ma:contentTypeVersion="17" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e787fa9c9cb978e1d00e8cc5d4e605d2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="31d8624d-d3e1-4449-addd-518bfa42d279" xmlns:ns3="637d3f4c-beee-42dd-a17b-93f7589025e5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="369004915ca410f163a62304f925ff92" ns2:_="" ns3:_="">
     <xsd:import namespace="31d8624d-d3e1-4449-addd-518bfa42d279"/>
@@ -3142,32 +3131,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6056489-A7A4-4445-AFC5-87E5586E5E93}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="637d3f4c-beee-42dd-a17b-93f7589025e5"/>
-    <ds:schemaRef ds:uri="31d8624d-d3e1-4449-addd-518bfa42d279"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B3AD83-9986-4E71-995F-A94C1CED6EB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="637d3f4c-beee-42dd-a17b-93f7589025e5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="31d8624d-d3e1-4449-addd-518bfa42d279">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B249E2D-022F-440D-B037-6C32F5252DA3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3184,4 +3168,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B3AD83-9986-4E71-995F-A94C1CED6EB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6056489-A7A4-4445-AFC5-87E5586E5E93}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="637d3f4c-beee-42dd-a17b-93f7589025e5"/>
+    <ds:schemaRef ds:uri="31d8624d-d3e1-4449-addd-518bfa42d279"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>